<commit_message>
refactor: AI finetune preserves formatting, remove Data Map, UI cleanup
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project-Documents/officialtestsheets/safetyKPIOrgB.xlsx
+++ b/Project-Documents/officialtestsheets/safetyKPIOrgB.xlsx
@@ -10,31 +10,22 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARD" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
   </externalReferences>
   <definedNames>
     <definedName name="AlBahahProvince">Dropdown!$AG$2:$AG$4</definedName>
     <definedName name="AlJoufProvince">Dropdown!$AH$2:$AH$3</definedName>
     <definedName name="AlMadinahProvince">Dropdown!$AJ$2:$AJ$4</definedName>
     <definedName name="AlQassimProvince">Dropdown!$AI$2:$AI$4</definedName>
-    <definedName name="Anticipated_Variation" localSheetId="2">'[1]Construction Cost Report'!$H$12</definedName>
-    <definedName name="Anticipated_Variation" localSheetId="1">'[1]Construction Cost Report'!$H$12</definedName>
     <definedName name="Anticipated_Variation">#REF!</definedName>
-    <definedName name="Approved_Additional_Budget" localSheetId="2">'[1]Construction Cost Report'!$H$4</definedName>
-    <definedName name="Approved_Additional_Budget" localSheetId="1">'[1]Construction Cost Report'!$H$4</definedName>
     <definedName name="Approved_Additional_Budget">#REF!</definedName>
     <definedName name="AsirProvince">Dropdown!$AK$2:$AK$6</definedName>
     <definedName name="Budget_For_Current_Commitment">#REF!</definedName>
-    <definedName name="Current_Approved_Budget" localSheetId="2">'[1]Construction Cost Report'!$H$5</definedName>
-    <definedName name="Current_Approved_Budget" localSheetId="1">'[1]Construction Cost Report'!$H$5</definedName>
     <definedName name="Current_Approved_Budget">#REF!</definedName>
-    <definedName name="Current_Commitment" localSheetId="2">'[1]Construction Cost Report'!$H$9</definedName>
-    <definedName name="Current_Commitment" localSheetId="1">'[1]Construction Cost Report'!$H$9</definedName>
     <definedName name="Current_Commitment">#REF!</definedName>
-    <definedName name="Early_Warning" localSheetId="2">'[1]Construction Cost Report'!$H$11</definedName>
-    <definedName name="Early_Warning" localSheetId="1">'[1]Construction Cost Report'!$H$11</definedName>
     <definedName name="Early_Warning">#REF!</definedName>
     <definedName name="EasternProvince">Dropdown!$AL$2:$AL$15</definedName>
     <definedName name="Education">Dropdown!$T$2:$T$7</definedName>
@@ -48,8 +39,6 @@
     <definedName name="NajranProvince">Dropdown!$AP$2:$AP$3</definedName>
     <definedName name="NorthernBordersProvince">Dropdown!$AQ$2:$AQ$5</definedName>
     <definedName name="Office">Dropdown!$Q$2:$Q$4</definedName>
-    <definedName name="Original_Budget" localSheetId="2">'[1]Construction Cost Report'!$H$3</definedName>
-    <definedName name="Original_Budget" localSheetId="1">'[1]Construction Cost Report'!$H$3</definedName>
     <definedName name="Original_Budget">#REF!</definedName>
     <definedName name="OtherAccommodation">Dropdown!$X$2:$X$3</definedName>
     <definedName name="Parking">Dropdown!$Y$2</definedName>
@@ -58,13 +47,25 @@
     <definedName name="RiyadhProvince">Dropdown!$AR$2:$AR$12</definedName>
     <definedName name="SocialInfrastructure">Dropdown!$V$2:$V$8</definedName>
     <definedName name="TabukProvince">Dropdown!$AS$2:$AS$3</definedName>
-    <definedName name="Total_Original_Awarded_Contracts" localSheetId="2">'[1]Construction Cost Report'!$H$7</definedName>
-    <definedName name="Total_Original_Awarded_Contracts" localSheetId="1">'[1]Construction Cost Report'!$H$7</definedName>
     <definedName name="Total_Original_Awarded_Contracts">#REF!</definedName>
     <definedName name="TransportLogisticIndustrial">Dropdown!$W$2:$W$10</definedName>
+    <definedName name="Variation_Orders">#REF!</definedName>
+    <definedName name="Anticipated_Variation" localSheetId="1">'[1]Construction Cost Report'!$H$12</definedName>
+    <definedName name="Approved_Additional_Budget" localSheetId="1">'[1]Construction Cost Report'!$H$4</definedName>
+    <definedName name="Current_Approved_Budget" localSheetId="1">'[1]Construction Cost Report'!$H$5</definedName>
+    <definedName name="Current_Commitment" localSheetId="1">'[1]Construction Cost Report'!$H$9</definedName>
+    <definedName name="Early_Warning" localSheetId="1">'[1]Construction Cost Report'!$H$11</definedName>
+    <definedName name="Original_Budget" localSheetId="1">'[1]Construction Cost Report'!$H$3</definedName>
+    <definedName name="Total_Original_Awarded_Contracts" localSheetId="1">'[1]Construction Cost Report'!$H$7</definedName>
+    <definedName name="Variation_Orders" localSheetId="1">'[1]Construction Cost Report'!$H$8</definedName>
+    <definedName name="Anticipated_Variation" localSheetId="2">'[1]Construction Cost Report'!$H$12</definedName>
+    <definedName name="Approved_Additional_Budget" localSheetId="2">'[1]Construction Cost Report'!$H$4</definedName>
+    <definedName name="Current_Approved_Budget" localSheetId="2">'[1]Construction Cost Report'!$H$5</definedName>
+    <definedName name="Current_Commitment" localSheetId="2">'[1]Construction Cost Report'!$H$9</definedName>
+    <definedName name="Early_Warning" localSheetId="2">'[1]Construction Cost Report'!$H$11</definedName>
+    <definedName name="Original_Budget" localSheetId="2">'[1]Construction Cost Report'!$H$3</definedName>
+    <definedName name="Total_Original_Awarded_Contracts" localSheetId="2">'[1]Construction Cost Report'!$H$7</definedName>
     <definedName name="Variation_Orders" localSheetId="2">'[1]Construction Cost Report'!$H$8</definedName>
-    <definedName name="Variation_Orders" localSheetId="1">'[1]Construction Cost Report'!$H$8</definedName>
-    <definedName name="Variation_Orders">#REF!</definedName>
   </definedNames>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
@@ -194,7 +195,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -267,8 +268,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.7999816888943144"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="39">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -742,6 +748,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -754,7 +782,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -1014,6 +1042,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2161,7 +2202,7 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" algorithmName="SHA-512" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" saltValue="/O3lGCmLZSLE293neApo1A==" formatRows="1" sort="1" spinCount="100000" hashValue="4/OMqn/JN28C38PSF6AJlZboViN/FzEY3LkHJU9y/nJUl7DFloR2MWwww+FlY+0ldrmVINVzWdPY45bqcbIy/A=="/>
   <dataValidations count="1">
-    <dataValidation sqref="D4:D5" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="date" operator="greaterThanOrEqual">
+    <dataValidation sqref="D4:D5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="date" operator="greaterThanOrEqual">
       <formula1>43831</formula1>
     </dataValidation>
   </dataValidations>
@@ -25123,12 +25164,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="N8:O8"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="L8:M8"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="D4:E6"/>
-    <mergeCell ref="N8:O8"/>
     <mergeCell ref="C4:C6"/>
-    <mergeCell ref="L8:M8"/>
   </mergeCells>
   <conditionalFormatting sqref="R10">
     <cfRule type="cellIs" priority="42" operator="greaterThan" dxfId="0">
@@ -25371,10 +25412,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="Q38:Q106 F38:P1006 F37:H37 P11:Q12 L17:Q24 L35:Q35 L26:Q28 L37:Q37 L11:O11 F17:H20 F11:H11 F23:H24 F26:H28 F35:H35 K10:K37 F32:H32 L32:Q32" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="F11:H11 F17:H20 F23:H24 F26:H28 F32:H32 F35:H35 F37:H37 F38:P1006 K10:K37 L11:O11 L17:Q24 L26:Q28 L32:Q32 L35:Q35 L37:Q37 P11:Q12 Q38:Q106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="R44:R1006 R10:R39" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="decimal">
+    <dataValidation sqref="R10:R39 R44:R1006" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="decimal">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -25653,34 +25694,34 @@
         </is>
       </c>
       <c r="F10" s="77" t="n">
-        <v>125000</v>
+        <v>130000</v>
       </c>
       <c r="G10" s="76" t="n">
-        <v>124800</v>
+        <v>129700</v>
       </c>
       <c r="H10" s="76" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="76" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="K10" s="76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="76" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="M10" s="76" t="n">
-        <v>215</v>
+        <v>195</v>
       </c>
       <c r="N10" s="76" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O10" s="76" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" ht="16" customFormat="1" customHeight="1" s="17">
@@ -25694,10 +25735,10 @@
         </is>
       </c>
       <c r="F11" s="78" t="n">
-        <v>88000</v>
+        <v>85000</v>
       </c>
       <c r="G11" s="76" t="n">
-        <v>87900</v>
+        <v>84800</v>
       </c>
       <c r="H11" s="76" t="n">
         <v>0</v>
@@ -25709,19 +25750,19 @@
         <v>0</v>
       </c>
       <c r="K11" s="76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L11" s="76" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M11" s="76" t="n">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="N11" s="76" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O11" s="76" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="1" s="17">
@@ -25735,7 +25776,7 @@
         </is>
       </c>
       <c r="F12" s="78" t="n">
-        <v>42000</v>
+        <v>40000</v>
       </c>
       <c r="G12" s="76" t="n">
         <v>42000</v>
@@ -25750,19 +25791,19 @@
         <v>0</v>
       </c>
       <c r="K12" s="76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" s="76" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="M12" s="76" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="N12" s="76" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O12" s="76" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="1" s="17">
@@ -25906,13 +25947,13 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="D4:F6"/>
     <mergeCell ref="D3:F3"/>
     <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D4:F6"/>
-    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G10:N15 F13:F15" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="F13:F15 G10:N15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -27367,4 +27408,272 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B3:P6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5.16" customWidth="1" min="1" max="1"/>
+    <col width="23.33" customWidth="1" min="2" max="2"/>
+    <col width="27.5" customWidth="1" min="3" max="3"/>
+    <col width="15.66" customWidth="1" min="4" max="4"/>
+    <col width="25.66" customWidth="1" min="5" max="5"/>
+    <col width="15.66" customWidth="1" min="6" max="6"/>
+    <col width="33.66" customWidth="1" min="7" max="7"/>
+    <col width="15.66" customWidth="1" min="8" max="8"/>
+    <col width="25.66" customWidth="1" min="9" max="9"/>
+    <col width="18.66" customWidth="1" min="10" max="10"/>
+    <col width="28.16" customWidth="1" min="11" max="11"/>
+    <col width="15.66" customWidth="1" min="12" max="12"/>
+    <col width="19.5" customWidth="1" min="13" max="13"/>
+    <col width="15.66" customWidth="1" min="14" max="14"/>
+    <col width="27.33" customWidth="1" min="15" max="15"/>
+    <col width="14.16" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="3" ht="153.5" customHeight="1">
+      <c r="B3" s="97" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="C3" s="98" t="inlineStr">
+        <is>
+          <t>A work-related incident or ill-health resulting in the death of one or more persons within the project.</t>
+        </is>
+      </c>
+      <c r="D3" s="98" t="n"/>
+      <c r="E3" s="98" t="inlineStr">
+        <is>
+          <t>An incident or ill-health resulting in a person being unable to carry work for one or more full workday or shift, not including the day or first shift of the incident or start of the ill-health.</t>
+        </is>
+      </c>
+      <c r="F3" s="98" t="n"/>
+      <c r="G3" s="98" t="inlineStr">
+        <is>
+          <t>Measures work-related injury or illness that requires medical treatment beyond first aid. This means that the injury or illness needs care from a professional healthcare provider, such as a physician or qualified paramedic, but does not result in time off work or restricted 
+work duties. (Total incidents from project inception to the current date).</t>
+        </is>
+      </c>
+      <c r="H3" s="98" t="n"/>
+      <c r="I3" s="98" t="inlineStr">
+        <is>
+          <t>Captures the total near miss incidents or situation that could have resulted in an injury, illness, or damage, but did not, due to luck or intervention. (Total incidents from project inception to the current date).</t>
+        </is>
+      </c>
+      <c r="J3" s="98" t="n"/>
+      <c r="K3" s="98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Captures the total number of safety observations reported in a project from its inception till its current date. </t>
+        </is>
+      </c>
+      <c r="L3" s="98" t="n"/>
+      <c r="M3" s="98" t="inlineStr">
+        <is>
+          <t>Captures the total number of documented project site safety walks conducted by leadership (CEO, CDO, project executives) from project inception till current date.</t>
+        </is>
+      </c>
+      <c r="N3" s="98" t="n"/>
+      <c r="O3" s="98" t="inlineStr">
+        <is>
+          <t>Captures the total number of formal HSE rewards, and recognitions provided to contractors &amp; individuals as an appreciation for their high performance. 
+(During this reporting month)</t>
+        </is>
+      </c>
+      <c r="P3" s="98" t="n"/>
+    </row>
+    <row r="4" ht="106.5" customHeight="1">
+      <c r="C4" s="98" t="inlineStr">
+        <is>
+          <t>1. 0 :  Score 100%
+2. &gt; 0 and ≤ 0.01: Score 90%
+3. 0.01 and ≤ 0.05: Score 80
+4. 0.05 and ≤ 0.1: Score 070%
+5. &gt; 0.1: Score Zero</t>
+        </is>
+      </c>
+      <c r="D4" s="98" t="n"/>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>0 :  Score 100%
+&gt; 0 and ≤ 0.04: Score 90%
+&gt; 0.04 and ≤ 0.1: Score 80%
+&gt; 0.1 and ≤ 0.2: Score 70%
+&gt; 0.2: Score Zero</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="n"/>
+      <c r="G4" s="98" t="inlineStr">
+        <is>
+          <t>0 :  Score 100%
+&gt; 0 and ≤ 0.045: Score 90%
+&gt; 0.045 and ≤ 0.09: Score 80%
+&gt; 0.09 and ≤ 0.15: Score 70%
+&gt; 0.15: Score Zero</t>
+        </is>
+      </c>
+      <c r="H4" s="98" t="n"/>
+      <c r="I4" s="98" t="inlineStr">
+        <is>
+          <t>&gt; 5.0: Score 100%
+3.0 - 5.0: Score 90%
+1.0 - 3.0: Score 80%
+&lt; 1.0: Score 70%
+0: Score Zero</t>
+        </is>
+      </c>
+      <c r="J4" s="98" t="n"/>
+      <c r="K4" s="98" t="inlineStr">
+        <is>
+          <t>&gt; 100: Score 100%
+80 - 100: Score 90%
+60 - 80: Score 80%
+40 - 60: Score 70%
+&lt; 40: Score Zero</t>
+        </is>
+      </c>
+      <c r="L4" s="98" t="n"/>
+      <c r="M4" s="98" t="inlineStr">
+        <is>
+          <t>&gt; 7.0: Score 100%
+5.0 - 7.0: Score 95%
+3.0 - 5.0: Score 90%
+2.0 - 3.0: Score 85%
+&lt; 2.0: Score 80%
+0: Score Zero</t>
+        </is>
+      </c>
+      <c r="N4" s="98" t="n"/>
+      <c r="O4" s="98" t="inlineStr">
+        <is>
+          <t>&gt; 0.4: Score 100%
+0.3 - 0.4: Score 95% 
+0.2 - 0.3 : Score 90% 
+0.1 - 0.2: Score 85%
+&lt; 0.1 : Score 80%
+0: Score Zero</t>
+        </is>
+      </c>
+      <c r="P4" s="98" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="C5" s="97" t="inlineStr">
+        <is>
+          <t>No. of Fatality in the project</t>
+        </is>
+      </c>
+      <c r="D5" s="98" t="n"/>
+      <c r="E5" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lost Time Injury incidents </t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="n"/>
+      <c r="G5" s="98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Recordable 
+Incident </t>
+        </is>
+      </c>
+      <c r="H5" s="98" t="n"/>
+      <c r="I5" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Near Miss incidents </t>
+        </is>
+      </c>
+      <c r="J5" s="98" t="n"/>
+      <c r="K5" s="97" t="inlineStr">
+        <is>
+          <t>Total Safety Observations</t>
+        </is>
+      </c>
+      <c r="L5" s="98" t="n"/>
+      <c r="M5" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Leadership safety walks conducted </t>
+        </is>
+      </c>
+      <c r="N5" s="98" t="n"/>
+      <c r="O5" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total number of Recognitions &amp; rewards </t>
+        </is>
+      </c>
+      <c r="P5" s="98" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="99" t="inlineStr">
+        <is>
+          <t>Ardara</t>
+        </is>
+      </c>
+      <c r="C6" s="100">
+        <f>ARD!$H$17</f>
+        <v/>
+      </c>
+      <c r="D6" s="101">
+        <f t="array" ref="D6">_xlfn.IFS(C6=0,100%,AND(C6&gt;0,C6&lt;=0.01),90%,AND(C6&gt;0.01,C6&lt;=0.05),80%,AND(C6&gt;0.05,C6&lt;=0.1),70%,C6&gt;0.1,0%)</f>
+        <v/>
+      </c>
+      <c r="E6" s="100">
+        <f>ARD!$I$17</f>
+        <v/>
+      </c>
+      <c r="F6" s="101">
+        <f t="array" ref="F6">_xlfn.IFS(E6=0,100%,AND(E6&gt;0,E6&lt;=0.04),90%,AND(E6&gt;0.04,E6&lt;=0.1),80%,AND(E6&gt;0.1,E6&lt;=0.2),70%,E6&gt;0.2,0%)</f>
+        <v/>
+      </c>
+      <c r="G6" s="100">
+        <f>ARD!K17</f>
+        <v/>
+      </c>
+      <c r="H6" s="101">
+        <f t="array" ref="H6">_xlfn.IFS(G6=0,100%,AND(G6&gt;0,G6&lt;=0.045),90%,AND(G6&gt;0.045,G6&lt;=0.09),80%,AND(G6&gt;0.09,G6&lt;=0.15),70%,G6&gt;0.15,0%)</f>
+        <v/>
+      </c>
+      <c r="I6" s="100">
+        <f>ARD!L17</f>
+        <v/>
+      </c>
+      <c r="J6" s="101">
+        <f t="array" ref="J6">_xlfn.IFS(I6=0,0%,AND(I6&gt;30,I6&lt;=40),90%,AND(I6&gt;20,I6&lt;=0.3),80%,AND(I6&gt;10,I6&lt;=20),70%,AND(I6&lt;10),70%,I6&gt;40,100%)</f>
+        <v/>
+      </c>
+      <c r="K6" s="100">
+        <f>ARD!M17</f>
+        <v/>
+      </c>
+      <c r="L6" s="101">
+        <f t="array" ref="L6">_xlfn.IFS(K6&gt;100,100%,AND(K6&gt;80,K6&lt;=100),90%,AND(K6&gt;60,G6&lt;=80),80%,AND(K6&gt;40,G6&lt;=60),70%,K6&lt;40,0%)</f>
+        <v/>
+      </c>
+      <c r="M6" s="100">
+        <f>ARD!N17</f>
+        <v/>
+      </c>
+      <c r="N6" s="101">
+        <f t="array" ref="N6">_xlfn.IFS(M6=0,0%,AND(M6&gt;5,M6&lt;=7),95%,AND(M6&gt;3,M6&lt;=5),90%,AND(M6&gt;2,M6&lt;=3),85%,AND(M6&lt;2),80%,M6&gt;7,100%)</f>
+        <v/>
+      </c>
+      <c r="O6" s="100">
+        <f>ARD!O17</f>
+        <v/>
+      </c>
+      <c r="P6" s="101">
+        <f t="array" ref="P6">_xlfn.IFS(O6=0,0%,AND(O6&gt;0.3,O6&lt;=0.4),95%,AND(O6&gt;0.2,O6&lt;=0.3),90%,AND(O6&gt;0.1,O6&lt;=0.2),85%,AND(O6&lt;0.1),80%,O6&gt;0.4,100%)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:B5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>